<commit_message>
fix the turnover issue
</commit_message>
<xml_diff>
--- a/backend/exports/All_Extracted_Leads.xlsx
+++ b/backend/exports/All_Extracted_Leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__lead_export_mapping__" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LeadCommonImportDTO'!$A$1:$P$156</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LeadCommonImportDTO'!$A$1:$P$177</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -930,7 +930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P156"/>
+  <dimension ref="A1:P177"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.88671875" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col width="11.109375" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -5091,9 +5091,6 @@
           <t>adityaautocomponents</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr"/>
-      <c r="D135" t="inlineStr"/>
-      <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
           <t>094483 74377</t>
@@ -5114,17 +5111,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="J135" t="inlineStr"/>
-      <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr">
         <is>
           <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M135" t="inlineStr"/>
-      <c r="N135" t="inlineStr"/>
-      <c r="O135" t="inlineStr"/>
-      <c r="P135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5137,9 +5128,6 @@
           <t>GLOBAL AUTO COMPONENTS // MOLEX, JST/TE, TYCO, AMP, HRS, SUMITOMO, YAZAKI , KET , SAMTEC, 3M</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr"/>
-      <c r="D136" t="inlineStr"/>
-      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
           <t>095139 69966</t>
@@ -5160,17 +5148,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr"/>
-      <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr">
         <is>
           <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M136" t="inlineStr"/>
-      <c r="N136" t="inlineStr"/>
-      <c r="O136" t="inlineStr"/>
-      <c r="P136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5183,9 +5165,6 @@
           <t>Hamson Automotive</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr"/>
-      <c r="D137" t="inlineStr"/>
-      <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
           <t>+918078102515</t>
@@ -5206,17 +5185,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr"/>
-      <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr">
         <is>
           <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M137" t="inlineStr"/>
-      <c r="N137" t="inlineStr"/>
-      <c r="O137" t="inlineStr"/>
-      <c r="P137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -5229,9 +5202,6 @@
           <t>Bangalore Auto Parts</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr"/>
-      <c r="D138" t="inlineStr"/>
-      <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
           <t>+91 8618713187</t>
@@ -5267,10 +5237,6 @@
           <t>unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M138" t="inlineStr"/>
-      <c r="N138" t="inlineStr"/>
-      <c r="O138" t="inlineStr"/>
-      <c r="P138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -5283,21 +5249,16 @@
           <t>Maruthi Auto Components</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr"/>
-      <c r="D139" t="inlineStr"/>
-      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>082961 13423</t>
         </is>
       </c>
-      <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr">
         <is>
           <t>2G67+F6P, 8th Cross Rd</t>
         </is>
       </c>
-      <c r="I139" t="inlineStr"/>
       <c r="J139" t="inlineStr">
         <is>
           <t>29AFWPG9138A1Z4</t>
@@ -5313,10 +5274,6 @@
           <t>unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
         </is>
       </c>
-      <c r="M139" t="inlineStr"/>
-      <c r="N139" t="inlineStr"/>
-      <c r="O139" t="inlineStr"/>
-      <c r="P139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -5329,11 +5286,6 @@
           <t>dC Auto Parts Pvt. Limited</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr"/>
-      <c r="D140" t="inlineStr"/>
-      <c r="E140" t="inlineStr"/>
-      <c r="F140" t="inlineStr"/>
-      <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr">
         <is>
           <t>Pune - Bengaluru Hwy</t>
@@ -5344,17 +5296,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr">
         <is>
           <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M140" t="inlineStr"/>
-      <c r="N140" t="inlineStr"/>
-      <c r="O140" t="inlineStr"/>
-      <c r="P140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5367,7 +5313,6 @@
           <t>Toyota Industries Engine India Private Limited</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
           <t>Mr. Keiichi Ido</t>
@@ -5378,7 +5323,6 @@
           <t>Managing Director</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
           <t>tiei@tiei.toyota-industries.com</t>
@@ -5409,10 +5353,6 @@
           <t>unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M141" t="inlineStr"/>
-      <c r="N141" t="inlineStr"/>
-      <c r="O141" t="inlineStr"/>
-      <c r="P141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5425,11 +5365,6 @@
           <t>GLOBAL AUTO PARTS</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr"/>
-      <c r="D142" t="inlineStr"/>
-      <c r="E142" t="inlineStr"/>
-      <c r="F142" t="inlineStr"/>
-      <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
           <t>119/9, Lalbagh Fort Rd</t>
@@ -5455,10 +5390,6 @@
           <t>unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M142" t="inlineStr"/>
-      <c r="N142" t="inlineStr"/>
-      <c r="O142" t="inlineStr"/>
-      <c r="P142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -5471,9 +5402,6 @@
           <t>Gi Auto Private Limited</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr"/>
-      <c r="D143" t="inlineStr"/>
-      <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
           <t>080 2525 2437</t>
@@ -5494,17 +5422,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
       <c r="L143" t="inlineStr">
         <is>
           <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M143" t="inlineStr"/>
-      <c r="N143" t="inlineStr"/>
-      <c r="O143" t="inlineStr"/>
-      <c r="P143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5517,32 +5439,21 @@
           <t>Top Level Car Accessories</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr"/>
-      <c r="D144" t="inlineStr"/>
-      <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
           <t>089518 43398</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr">
         <is>
           <t>Tq, near Nandishwara theater Tent</t>
         </is>
       </c>
-      <c r="I144" t="inlineStr"/>
-      <c r="J144" t="inlineStr"/>
-      <c r="K144" t="inlineStr"/>
       <c r="L144" t="inlineStr">
         <is>
           <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
         </is>
       </c>
-      <c r="M144" t="inlineStr"/>
-      <c r="N144" t="inlineStr"/>
-      <c r="O144" t="inlineStr"/>
-      <c r="P144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5555,28 +5466,16 @@
           <t>Tata Yazaki Auto Comp Limited</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr"/>
-      <c r="D145" t="inlineStr"/>
-      <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr"/>
-      <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr">
         <is>
           <t>319(p, Bommasandra Jigani Link Rd</t>
         </is>
       </c>
-      <c r="I145" t="inlineStr"/>
-      <c r="J145" t="inlineStr"/>
-      <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr">
         <is>
           <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
         </is>
       </c>
-      <c r="M145" t="inlineStr"/>
-      <c r="N145" t="inlineStr"/>
-      <c r="O145" t="inlineStr"/>
-      <c r="P145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -5589,9 +5488,6 @@
           <t>Avinash Automobiles</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr"/>
-      <c r="D146" t="inlineStr"/>
-      <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
         <is>
           <t>099458 88887</t>
@@ -5607,18 +5503,11 @@
           <t>H. NO. 944, OTUR ROAD TALUKA KALWAN, DIST. NASHIK KALWAN Nashik Maharashtra - 425001</t>
         </is>
       </c>
-      <c r="I146" t="inlineStr"/>
-      <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr"/>
       <c r="L146" t="inlineStr">
         <is>
           <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
         </is>
       </c>
-      <c r="M146" t="inlineStr"/>
-      <c r="N146" t="inlineStr"/>
-      <c r="O146" t="inlineStr"/>
-      <c r="P146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5631,10 +5520,6 @@
           <t>Nexteer Automotive</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr"/>
-      <c r="D147" t="inlineStr"/>
-      <c r="E147" t="inlineStr"/>
-      <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
         <is>
           <t>nexteer.contact@nexteer.com</t>
@@ -5650,17 +5535,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
       <c r="L147" t="inlineStr">
         <is>
           <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M147" t="inlineStr"/>
-      <c r="N147" t="inlineStr"/>
-      <c r="O147" t="inlineStr"/>
-      <c r="P147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5673,10 +5552,6 @@
           <t>jigani</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr"/>
-      <c r="D148" t="inlineStr"/>
-      <c r="E148" t="inlineStr"/>
-      <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
         <is>
           <t>papannajigani@gmail.com</t>
@@ -5692,17 +5567,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
       <c r="L148" t="inlineStr">
         <is>
           <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M148" t="inlineStr"/>
-      <c r="N148" t="inlineStr"/>
-      <c r="O148" t="inlineStr"/>
-      <c r="P148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5715,28 +5584,16 @@
           <t>Fine Components and Tools Pvt Ltd Unit 1 Gate No.02</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr"/>
-      <c r="D149" t="inlineStr"/>
-      <c r="E149" t="inlineStr"/>
-      <c r="F149" t="inlineStr"/>
-      <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
           <t>31, Bommasandra Jigani Link Rd</t>
         </is>
       </c>
-      <c r="I149" t="inlineStr"/>
-      <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
       <c r="L149" t="inlineStr">
         <is>
           <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
         </is>
       </c>
-      <c r="M149" t="inlineStr"/>
-      <c r="N149" t="inlineStr"/>
-      <c r="O149" t="inlineStr"/>
-      <c r="P149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5749,15 +5606,11 @@
           <t>Viana AutoZone</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr"/>
-      <c r="D150" t="inlineStr"/>
-      <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
           <t>086183 90776</t>
         </is>
       </c>
-      <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr">
         <is>
           <t>Jigani 2A, Plot 47</t>
@@ -5768,17 +5621,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr">
         <is>
           <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M150" t="inlineStr"/>
-      <c r="N150" t="inlineStr"/>
-      <c r="O150" t="inlineStr"/>
-      <c r="P150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5791,7 +5638,6 @@
           <t>Lamda Components Pvt Ltd.</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr">
         <is>
           <t>Lamda Components</t>
@@ -5822,17 +5668,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
       <c r="L151" t="inlineStr">
         <is>
           <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M151" t="inlineStr"/>
-      <c r="N151" t="inlineStr"/>
-      <c r="O151" t="inlineStr"/>
-      <c r="P151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5845,9 +5685,6 @@
           <t>Sansera Engineering</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr"/>
-      <c r="D152" t="inlineStr"/>
-      <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr">
         <is>
           <t>080 2783 9309</t>
@@ -5868,17 +5705,11 @@
           <t>Bangalore</t>
         </is>
       </c>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
       <c r="L152" t="inlineStr">
         <is>
           <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M152" t="inlineStr"/>
-      <c r="N152" t="inlineStr"/>
-      <c r="O152" t="inlineStr"/>
-      <c r="P152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5891,32 +5722,21 @@
           <t>Sri Varalakshmi Auto Components Pvt. Ltd.</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr"/>
-      <c r="D153" t="inlineStr"/>
-      <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
           <t>099720 36978</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
           <t>4th &amp;, No. 2 &amp; 3, 5th Cross, near Sunkadakatte</t>
         </is>
       </c>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
       <c r="L153" t="inlineStr">
         <is>
           <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
         </is>
       </c>
-      <c r="M153" t="inlineStr"/>
-      <c r="N153" t="inlineStr"/>
-      <c r="O153" t="inlineStr"/>
-      <c r="P153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5929,15 +5749,11 @@
           <t>AMJ Auto Components</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr"/>
-      <c r="D154" t="inlineStr"/>
-      <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr">
         <is>
           <t>098455 24875</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
           <t>65/38, Rangappa Layout, 2nd cross, Post</t>
@@ -5948,17 +5764,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
       <c r="L154" t="inlineStr">
         <is>
           <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M154" t="inlineStr"/>
-      <c r="N154" t="inlineStr"/>
-      <c r="O154" t="inlineStr"/>
-      <c r="P154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -5971,9 +5781,6 @@
           <t>Ace Forge Private Limited</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr"/>
-      <c r="D155" t="inlineStr"/>
-      <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
           <t>063639 22746</t>
@@ -5994,17 +5801,11 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr">
         <is>
           <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
         </is>
       </c>
-      <c r="M155" t="inlineStr"/>
-      <c r="N155" t="inlineStr"/>
-      <c r="O155" t="inlineStr"/>
-      <c r="P155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -6017,35 +5818,696 @@
           <t>Modtech Engineering</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr"/>
-      <c r="D156" t="inlineStr"/>
-      <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr">
         <is>
           <t>098458 85811</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr">
         <is>
           <t>Bommasandra Jigani Link Rd, behind Omax auto 95</t>
         </is>
       </c>
-      <c r="I156" t="inlineStr"/>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
       <c r="L156" t="inlineStr">
         <is>
           <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
         </is>
       </c>
-      <c r="M156" t="inlineStr"/>
-      <c r="N156" t="inlineStr"/>
-      <c r="O156" t="inlineStr"/>
-      <c r="P156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Jaggi Industries</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Mr Sukhvinder Singh</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>080 4547 8560</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>B-62, Mayapuri Industrial Area, Phase-II,New Delhi - 110064, India</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>07AAEFJ9793R1Z8</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Rs. 5 Cr. to 25 Cr.</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Neerflow Pumps LLP</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>099110 04200</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>info@neerflow.com</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>C-83, Mayapuri Industrial Area, Phase-II 110064, New Delhi</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Indraprastha Gas Limited CNG Station</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>074289 44273</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Plot No. 4, Community Centre,, Sector 9, R K Puram, New Delhi - 110022</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>New Delhi</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>NARAYAN WATER PUMP &amp; Pressure Pump - Plumbers &amp; Electrician</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>092785 44293</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Sector-1, Pocket-00, book Depot Road, nearby Kanjhawala Road</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>TULFI Point-Sector 8 Petrol Pump</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>P43C+2P8</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>igl cng pump</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>P3HX+362</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Bharat Petroleum, Petrol Pump -Sanjeev Filling Station</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Fluid Frontliners</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Anurag Kalra</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>080 4389 1650</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>58, G.B Road, Shardhanad Marg, New Delhi - 110006, Delhi, India</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>07APQPK5379F1ZE</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>25 Cr</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>The Pump Factory</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>099908 05408</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Lakhiramchowk, opposite The Great Ashoka public school</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Police Petrol Pump Pitampura</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>1, Police Lines, near Marble Market</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Indane Petrol pump and cng station</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>P466+J2C</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Bharat Petroleum, Petrol Pump -Shaurya Bhushan Filling Station</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>RAM KRISHAN MARG DELHI</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Archana Trading Company (ATC)</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Micromulti Grease</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>098186 17872</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>info@archanatradingcompany.com</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Third Floor, back side, C-75</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Rattan Hose &amp; Engineering Works Pvt. Limited.</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>011 4709 6666</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>info@rattanhose.com</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>C-67, Mayapuri Industrial Area, Phase-II, New Delhi-110064, (India)</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>New Delhi</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>GRECO CNG</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>098197 49380</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>A-14</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Ace Automation Engineers</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>011 4554 6564</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>oilcoolers@acefluidpower.com</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Compared to water cooling systems, air cooled oil coolers are easy to install, require less maintenance and are more cost effective. They are widely used in CNC machines, hydraulic power packs, gear boxes, presses, injection moulding machines and many other heavy duty applications. A good quality oil cooler helps in increasing machine life, reducing breakdown time and improving overall productivity., C-164, Mayapuri Industrial Area,, Phase II, New Delhi – 110064, India</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Hydmark Applicon</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>011 4511 4611</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>sales@hydmark.com</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>A- 5/4 &amp; 6/4, Phase- 2,, Mayapuri Industrial Area, New Delhi - 110064, India</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>IMMENSE VALVE INDIA PVT LTD</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>099672 45659</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>UNIT 805, CRESCENT BUSINESS SQUARE, opp. SJ STUDIO METRO, near SAKINAKA</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Maham Valves Automation</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>077388 53658</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>GLOBAL STEEL &amp; ENGINEERING</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>099301 95335</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>163, Dr. MG Mahimtura Marg</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>JHON VALVES EXIM INDIA (SS DAIRY FITTINGS AND SS DAIRY VALVES IN MUMBAI,PIPE FILTER,AMUL DRAIN TRAP,SS MANHOLE COVER)</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>093228 78406</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>sales@jhonvalves.com</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Regd.Office No 10 2nd Floor, Aman House</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P156"/>
+  <autoFilter ref="A1:P177"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
fix the gst and turnover
</commit_message>
<xml_diff>
--- a/backend/exports/All_Extracted_Leads.xlsx
+++ b/backend/exports/All_Extracted_Leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="__lead_export_mapping__" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LeadCommonImportDTO'!$A$1:$P$177</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LeadCommonImportDTO'!$A$1:$P$329</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -930,7 +930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P177"/>
+  <dimension ref="A1:P329"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.88671875" defaultRowHeight="12" customHeight="1"/>
   <cols>
     <col width="11.109375" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -943,7 +943,7 @@
     <col width="50" customWidth="1" style="2" min="8" max="8"/>
     <col width="29.21875" customWidth="1" style="2" min="9" max="9"/>
     <col width="20.5546875" customWidth="1" style="2" min="10" max="10"/>
-    <col width="25" customWidth="1" style="2" min="11" max="11"/>
+    <col width="28" customWidth="1" style="2" min="11" max="11"/>
     <col width="50" customWidth="1" style="2" min="12" max="12"/>
     <col width="15.5546875" customWidth="1" style="2" min="13" max="13"/>
     <col width="21.109375" customWidth="1" style="2" min="14" max="14"/>
@@ -6506,8 +6506,4797 @@
         </is>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>KVS Automatic Water Level Controller (Fully Automatic System)</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>080727 01588</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>No.1/1, S/S Complex, Thanjavur Rd</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>EASWARAN ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Ibrahim park back side, 1E, Jalal Kudiri Street, W Blvd Rd</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Vaidheswaran industries</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>094426 42839</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>SIDCO INDUSTRIAL ESTATE, B8</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>HVK Systems &amp; Marketing Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>0422 230 0039</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>1485, Trichy Rd, Behind Elgin Ultra</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Tiruchirappalli</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>KAMAK</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>091500 47571</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Passport office, Kamak Associates 148, Old, W Blvd Rd, opp. New SBI Siruthozlil Branch</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>HTC Pipes &amp; fittings</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>097909 45934</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Plot 91</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>SRI Energy, Inc.</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>25521905</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>SF.NO. 115/4A, Vadugapatti Village, Illupur Taluk, Pudukottai District</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Power Trans Engineering</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>86, 87</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>ELLEM Engineering</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>098431 52005</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Sf no 99/2A, 13C,Sree Maruthi industrial Estate,</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Christor Taps &amp; Fittings</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>094431 58717</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>lks tower, 127/2, W Blvd Rd</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Tiruchchirappalli</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>London Hardwares Shop Trichy</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>098656 01786</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Devar Hall, Water Tank Shopping Complex, GF 8, W Blvd Rd</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Tiruchchirappalli</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Salem Auto Parts</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>SALEM AUTO SOLUTIONS</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>088258 22655</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>No.132, Suramangalam Main Rd</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Salem</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Vikas Cars Accessories (All Car Accessories Dealer in Salem)</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>099947 99115</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>250/10, Meyyanur Main Rd</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Jagadamba Auto Agencies</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>J5X5+GM4</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>KM CAR DECORS</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>M4FM+H59, Meyyanur Main Rd</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Salem</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>SEM ENTERPRISES PVT LTD</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>0427 233 5277</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>SRI P. R AARCADE,, 230, Itteri Rd</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Salem</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Rollz Cars (Car A/C Spars &amp; Services &amp; Pre Owned Cars Buying/Selling)</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>096295 23223</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>226A, Omalur Main Rd</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Siyon auto consulting</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>095668 10888</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>MDR439</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Jeyam Cool Spares</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>073737 67626</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>145/3, VMR Nagar Rd, near ARRS theatre</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Mahalakshmi Auto Centre</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>0427 426 5486</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>64/4 New East Pullikuthi Street</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>JEM Indiaa</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>090922 06362</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Thandavarayan oil Mill Compound, 406-1, Suramangalam Main Rd</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Salem</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Racing Car Point</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>097912 71150</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>J4MF+QR7</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Mytvs Car Accessories - Car Parlour</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>#222, silver Arrow Complex, 4 Roads Piller No. S72, opp. Church</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>MSB ELECTRONIC INDUSTRIES</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>098427 55449</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>51/12 chennan krisha puram</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Hutaib Engineering Company</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>099445 72993</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>95 D.D ROAD, Old Bus Stand Rd, opp. SANGAM COMPLEX, near ALANKAR THEATRE</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Muthuraj Automobiles</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>0424 226 9309</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>35(25, Agilmedu 7th Streer</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Sree Meenakshi Auto Spares</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>099946 66885</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>18A/1 sathy Road, Municipal Colony Main Rd</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Sree Meenakshi Automobiles</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>094871 06885</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>82, Perundurai Rd, opp. to kvb bank</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>XTREMZ Bike Accessories</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>098425 83338</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Sathiya Street, 275/1, Municipal Colony Main Rd</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Amman Auto Parts</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>094433 58802</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>1st cross, Jai balaji Nagar, Naal Rd</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Tamilnadu Auto Stores</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>099655 22578</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>21/2, P.A. Complex Behind Parimalam Complex, Road, Periyanna St</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Vijay Car Care &amp; Decors in Erode | Car Accessories Shop in Erode | Car Wash in Erode | Multi Brand Car Accessories in Erode</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>098421 32068</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>147/2, Nasiyanur Rd</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Sri Giri Auto Stores</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>098423 92924</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>389/1, Visakan Tower, Perundurai Rd</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>A-Team Auto Spares</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>098423 26325</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>370/2A, Perundurai Rd, near Ambal Auto</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Sri Senthil Autos - Hero MotoCorp</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>092899 22135</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>134 B, Perundurai Rd</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>SHRI VIGNESH CAR JEWELS</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>098428 65000</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>135, Perundurai Rd, opp. Ambal auto</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>AAUDIO ONE ERODE</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>098423 73379</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>106/2, Perundurai Rd</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>THIYAGU AUTOMOTIVES ERODE</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>075027 53172</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>The Noble Motor (Noble Servece)</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>Perundurai Rd, near TPN hospital</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>River Service Perundurai Road</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>092402 21746</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>Building No: 314 / 2A2, Chinna Sengodampalayam, Perundurai Rd</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Vinayaka Tyress</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>099949 29494</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>236, Chinnamuthu Main St</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Montra Electric - Adharvaa Electric Autos, Erode</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>08071 639 009</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>No 1/568, Perundurai Road, Vallipurathanpalayam, beside Tractor Service Centre</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Ashok Leyland Dost Erode</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>063803 23280</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>13/2, Perundurai Rd</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>River Store Perundurai Road</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>092402 56420</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>Chinna Kaadu Thottam, No: 314/2A2, Perundurai Rd, near Veerappampalayam Bypass</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Kia Car Showroom - Pressana Kia Chinna Sengodampalayam, Erode</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>063844 44500</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>72/83, Sengodampalayam Rd</t>
+        </is>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Iswarya Cars</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>098425 37575</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>6, OA Ramasamy St</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Harris Car Covers</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>097503 82222</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>207, Perundurai Rd, near Sri Vari Arangam</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Erode</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Oragadam</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>swathilands@gmail.com</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Transindia Control Systems Pvt.Ltd.</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>040 2781 0199</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>tic@transindiacontrols.in</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>Anjuman Campus,, 1st Floor, Beside Anjuman Office,, 125. M.G.Road, Secunderabad - 500003</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Secunderabad</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>ALL-TEC ELECTRICAL ENGINEERS</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>098663 19925</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>201,5-2-437, Seven Hills Villa, Rashtrapati Rd, opp. Arya Samaj Building Office</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Jothi Batteries</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>099443 42723</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>4B, Sankara Naidu St</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Cuddalore Old Town</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Janakiram&amp;Co (2 Wheeler spares)</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>PQX6+R9H</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Swaraj Tractors - M/S Sree Sakthi Automobiles</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>08071 433 657</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>Shop No 3, Varsha Garden Imperial Road, Two Way Road, nearby Virudhachalam - Cuddalore Road</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Force Motors - Thangam Force</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>063840 01421</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>VSP Krishnamurthy Reddiyar Nagar, 5, Nellikuppam Main Rd</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Kubota Tractor - Pondy Agricultural Machinery</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>Shop No 3, Nellikuppam Main Rd, nearby Indianoil Petrol Pump</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>Cuddalore</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Royal Enfield Service Center - Rooster Automobiles</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>088795 17692</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>Chellankuppam, 9, Imperial Rd</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Cuddalore</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Exide Care - Sri Devi Agencies</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>080 6955 8971</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>No 2, Saravana Complex, Mohan Singh St</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>KTM Husqvarna Cuddalore</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>093558 34384</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Transture Solutions</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>080124 80157</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Sri Ram sewing machine</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>077083 90887</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>PQ8C+Q2V</t>
+        </is>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Kun Škoda Showroom</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>091769 49000</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>RS No 223/2B, Chidambaram Rd</t>
+        </is>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Murugan Electricals</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>094441 64334</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>10, S Park St</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Jai Mahaveer Electricals</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>098848 28022</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>No 126/10,Yadaval Street, Padi</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Electrical Control Panel</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>095511 72864</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>45GC+8HM, MM Ave 1st St</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Swaraj Motors</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>085470 54304</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>32ABPFM2499F1ZZ</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>18,217 Crore</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Govind Auto Spares</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>095444 42009</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>Puliyarthala, Ulloor - Akkulam Rd</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Thiruvananthapuram</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>MIDDLE EAST AUTO PARTS. PVT .LTD</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>085907 09144</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>Sasthamangalam Jct</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>Thiruvananthapuram</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Scrap vehicle buying</t>
+        </is>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Candour Auto Tech Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>096332 22927</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>VP II, 1148, Nettayam Rd</t>
+        </is>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Amba Automobiles</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>089214 40702</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>Thakaraparambu Road TC 28/1923, 1-6</t>
+        </is>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Phoenix Car Spa</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>085939 99392</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>TC 13/ 352 (1) M.K Building Periyamkodu PO</t>
+        </is>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Old Bike scrap buyer</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>094007 35896</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>Pathiripally - Choozhampala Rd, near guru Mandram</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Xtremers - Auto hub</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>089218 74366</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>TC 6/1345, S-25, Anupama Nagar Pongummod</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Kabeer Used Bike Parts</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>T.c 38 2100, Melancode St</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Royal Enfield - Subha Auto Wares</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>0471 247 3020</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>Sitarama Building TC 80/2788 Attakulangara, Sreevaraham - Muckolakkal Rd</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>S.S SCRAPS &amp; METALS MART</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>079073 64753</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>V M Auto Agencies</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>094475 35111</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>JX3X+M54 11th stone</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>Nedumangad</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>La Maison Citroën, Trivandrum</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>085939 77777</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>TC-91/1042-8, EVM Autokraft India Private Limited - Citroen, N H Byepass Venpalavattom, Kadakampally Rd</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Michelin Tyres - Travencore Wheel Club</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>097119 99124</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>TC 16/390, Indeevaram, Cotton Hill Rd</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Moto Avenue</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>083300 16943</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>LMS Junction, Union Tower</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Thiruvananthapuram</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Mahindra Cherukara Vehicles - SUV &amp; Commercial Vehicle Showroom</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>088799 31870</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>Thiruvananthapuram N H Bypass Road, near IOCL petrol pump, Thrimoorthy Nagar, Muttathara Thiruvana</t>
+        </is>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>HITEC VALVES</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>094448 62329</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>hitecvalves@vsnl.net</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>No.3, Part I TASS Industrial Estate, Ambattur, Chennai – 600098, India</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>HP VALVES &amp; FITTINGS INDIA PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>S. Harichandran</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>044 2625 2537</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>sales@hpvalvesindia.com</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>SP-133, SIDCO Industrial Estate, Ambattur, Chennai - 600058, Tamil Nadu, India</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Floport Valves Private Limited</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Mr. G. Hem Kumar</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>094440 55503</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>floportvalves@gmail.com</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>SP.29,AMBATTUR INDUSTRIALESTATE,AMBATTUR MADRAS-58 TAMILNADU, TAMILNADU, Tamil Nadu, India, 600058 - 600058</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>ValvTechnologies</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>7138600400</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>info@valv.com</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>PLOT NO. 65,FUNCTIONAL DEVELOPMENT, PLOTS FOR ELECTRICAL ELECTRONICS INDUSTRIES OMR, P, ERUNGUDI, Chennai, CHENNAI, Tamil Nadu, India, 600096 - 600096</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Sakthi Industries-Excel Valves</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>099629 95721</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>sakthivalves@gmail.com</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>Plot No.1, 10th Street, Kamarajar Road, TASS Industrial Estate, Ambattur, Chennai 600 098, INDIA</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>www.hussainenterprise.in</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>091502 97330</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>navkarinte@yahoo.co.in</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>188 (New No. 268), Linghi Chetty Street, Chennai - 600 001</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>FLUID VALVE CO KELLYS GODOWN</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>36PW+MG2</t>
+        </is>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>S. J. Industries</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>098403 50439</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>sales@analapumps.com</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>73, Tass Industrial Estate, Ambattur, Chennai - 600 098. Tamil Nadu, India</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Bharat Petroleum - Nironka Royal Agency</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>45C9+2G8</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Autocom Industries</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>4555+J8X.320</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>VBM ENGINEERING PRODUCTS</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Lachu Auto Traders</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>098406 40582</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>No.17,18,19 Lajapathy raj street,opp to town bus stand gandhipuram cbe-641012, near Town Busstand</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Thanukkodi Aditya Auto Stores</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>0422 423 2777</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>No 408, 411, Dr Nanjappa Rd</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>NEW RAJA TOOLS - AUTO GARAGE TOOLS COIMBATORE</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>098430 88854</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>NSP Complex, 180/ A/15, Dr Nanjappa Rd, opp. Royal Agencies Furniture</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Sun Motor Parts</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>089251 02864</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>M.S.Nagar, Podanur Main Rd</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Infinity Automobile Spares</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>082208 98350</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>SS Car Accessories</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>099409 49074</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>0pp Nayara Petrol Bunk, 915, Dr Alagappa Chettiar Rd</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Good Luck Motor Parts</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>093637 11882</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>5/164,Aringar Anna Nagar</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>South India Trading Agencies</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>098430 16110</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Parsns Trade Plaza, 156, Dr Nanjappa Rd</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>The Braap Shop</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>085080 55444</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>1233, Mettupalayam Main Rd, near Naga Sai Temple</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>GLOBAL MULTI TECH - Electric Vehicle Spares Wholesaler</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>063697 21254</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>1137-1138, Sukrawarpet St</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>AB pumps</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>099655 56165</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>9, 240C, Dr Nanjappa Rd</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Vasanthi mill</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>4848+6HV</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>33AADFV2078E1ZD</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>25 Cr</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>V S Auto Electricals</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>099940 53011</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>1/801, Palavanjipalayam Ring Rd, near Sakthi hospital Kadeswara plywoods, opposite Dharapuram Main Road</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Tirupur Jobs</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>099760 93012</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>2/400 Rajendran compound</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Thiru annamalaiyar air compressor motor sales and servicee</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>090955 95465</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>new bus stand back side, 58/1A Lucky Nagar, Sathi theatre road</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>sivakasi auto parts</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>086088 12597</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>333/1, Virudhunagar Main Rd, opposite mukesh honda</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Saraswati Automobiles</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>088383 39521</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Do. No. 792 Periya Karuppan Road Sivakasi Tamil Nadu 626123</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Sivakasi</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>29EYVPP3328B1ZZ</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>SRI VALATHTHI AMMAN AUTOS</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>099941 21288</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>872/D Sivanadiyan Complex Kamak Road</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Star Auto Parts</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>094866 39903</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>500A, Virudhunagar Main Rd, opp. railway station</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>27ACGPH2998J1Z4</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover could not be parsed; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>MS Moto central helmet and accessories</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>FQ5X+RRX</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>SRI BAGAWATHI AUTOMOBILES</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>098432 46699</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>6/3 Arun Sundari Complex</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Bismi car care</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>084385 02277</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>60AcharmanArnachalamRoad</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Sri raja auto spares</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>182/2, Vembakottai Rd</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Sivakasi</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Auto Dynamics-Continental Tyres</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>079 4344 4312</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>231/2, Thiruthangal Rd, near SFR COLLEGE</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>M K GRAND AUTOMOBILES, SIVAKASI - BOSCH CAR SERVICE</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>091500 80077</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>S.NO-54/8A3A, THAYILPATTI VILLAGE MADATHUPATTI, MAIN RAOD, near IOCL PETROL PUMP</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki ARENA (Meenakshi Autozone, Sivakasi, Tiruthangal Road)</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>080 6221 6609</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>819, Thiruthangal Rd</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>Sivakasi</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>33AAKCM3378A1ZO</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>₹186.71 Crore</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Anbu Two Wheeler Spares</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>394/1A1 ALAMARATHUPATTI ROAD, Virudhunagar Main Rd</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Bikecenter accessories</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>096777 82020</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>KAYYEM MOTORS</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>098421 54125</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>872B, Kamak Rd</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Haribala Auto Spares</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>FRJ7+X4V</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>mhadev auto mobiles</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>070142 33840</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>218, seethakathi middle street, near kamarajar park</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>33AZDPN2935P1Z0</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>Rs. 0 to 40 lakhs</t>
+        </is>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>SPEED AUTO CARE &amp; PARTS</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Sudharsan Garden, 1189/1A1A</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Devi Sri Motors</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>087781 33832</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>HITEC VALVES</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>094448 62329</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>hitecvalves@vsnl.net</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>No.3, Part I TASS Industrial Estate, Ambattur, Chennai – 600098, India</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>HP VALVES &amp; FITTINGS INDIA PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>S. Harichandran</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>044 2625 2537</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>sales@hpvalvesindia.com</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>SP-133, SIDCO Industrial Estate, Ambattur, Chennai - 600058, Tamil Nadu, India</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>33AACCH0510P1ZU</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>₹72.11 Crore</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Floport Valves Private Limited</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Mr. G. Hem Kumar</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>094440 55503</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>floportvalves@gmail.com</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>SP.29,AMBATTUR INDUSTRIALESTATE,AMBATTUR MADRAS-58 TAMILNADU, TAMILNADU, Tamil Nadu, India, 600058 - 600058</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>www.hussainenterprise.in</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>091502 97330</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>navkarinte@yahoo.co.in</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>188 (New No. 268), Linghi Chetty Street, Chennai - 600 001</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Sakthi Industries-Excel Valves</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>099629 95721</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>sakthivalves@gmail.com</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Plot No.1, 10th Street, Kamarajar Road, TASS Industrial Estate, Ambattur, Chennai 600 098, INDIA</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>FLUID VALVE CO KELLYS GODOWN</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>36PW+MG2</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Humifogg Systems – Humidifier Manufacturer in Coimbatore</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>098422 57593</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>sales@humifoggsystems.com</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Prevention of dryness, static discharge, and material degradation during storage, No:32, Indumaa Nagar, Vilankurichi Road, Near Cheranma Nagar, Coimbatore, Tamil Nadu 641035</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>33AAEFH1275J1ZI</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>5 - 25 Cr</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>COSMIC PUMPS / ANNAM INDUSTRIES</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>099525 17732</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Site No. 12, S.F No. 353/1, Cosmic Pumps Buildings,, Vinayagar Kovil Street, Neelikompalayam,, Coimbatore, Tamil Nadu 641033, India</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Sarah pumps</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>098944 18218</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>302, Samraj trade centre, vilankuruchi main road, peelamedu</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>AB pumps</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>099655 56165</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>9, 240C, Dr Nanjappa Rd</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Santhi Agencies: Authorized CRI Pumps</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>099945 89339</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>33EKKPS4955N1ZA</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>Rs. 40 lakhs to 1.5 Cr.</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>unverified: industry not supplied; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Hindustan Petroleum Corporation Limited</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>097875 33000</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>15644910@retail.hpcl.co.in</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>Coimbatore, Tamil Nadu - 641016</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>Coimbatore</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>₹4,414.48 Crore</t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>unverified: employee count unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>MG MEDITECH</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr"/>
+      <c r="D316" t="inlineStr"/>
+      <c r="E316" t="inlineStr"/>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>078389 48874</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>mgmeditechindia@gmail.com</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>Head Office: Oﬃce No. SK A-27, Sector-112, Noida, Gautam Dudh Nagar (Uttar pradesh-201301)</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr"/>
+      <c r="K316" t="inlineStr"/>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable; unverified: location could not be confirmed against the requested area</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr"/>
+      <c r="N316" t="inlineStr"/>
+      <c r="O316" t="inlineStr"/>
+      <c r="P316" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Medico Electrode</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr"/>
+      <c r="D317" t="inlineStr"/>
+      <c r="E317" t="inlineStr"/>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>0120 488 0600</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>Sales@MedicoElectrodes.com</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Medico Electrodes International Limited,, Plot 142A / 11,12 &amp; 29, Noida Special Economic Zone, Noida – 201305</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>09AAHCM4229K1Z5</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>₹601.5 Crore</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M317" t="inlineStr"/>
+      <c r="N317" t="inlineStr"/>
+      <c r="O317" t="inlineStr"/>
+      <c r="P317" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Vignaharta Enterprises Private Limited</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr"/>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Saket Agarwal</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>098769 78488</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>info@healthyjeenasikho.com</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>Whether you need a hospital bed, oxygen concentrator, CPAP/BiPAP machine, wheelchair, or patient monitor, we have it all!, 📍Noida Brand Store Google Location: Near Hanuman Murti, Sector-49, Noida, 201304</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>06AAECV9995Q1Z2</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>₹16.36 Crore</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M318" t="inlineStr"/>
+      <c r="N318" t="inlineStr"/>
+      <c r="O318" t="inlineStr"/>
+      <c r="P318" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>iLife Medical Devices Pvt Ltd, Noida Office</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr"/>
+      <c r="D319" t="inlineStr"/>
+      <c r="E319" t="inlineStr"/>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>0120 320 0663</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>CARE@ILIFEMEDICA.COM</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>7, Sector 63 Rd</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr"/>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>₹22.75 Crore</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr"/>
+      <c r="N319" t="inlineStr"/>
+      <c r="O319" t="inlineStr"/>
+      <c r="P319" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Divine Health Home Care</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr"/>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Moh Irshad</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>093551 00499</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>info@divinehealthathome.com</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>Gr. Noida West : 15A &amp; 22A, First Floor, Near Chunmun, Galaxy Blue Sapphire Plaza, Greater Noida West (Noida Extension), Uttar Pradesh 201301</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr"/>
+      <c r="K320" t="inlineStr"/>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr"/>
+      <c r="N320" t="inlineStr"/>
+      <c r="O320" t="inlineStr"/>
+      <c r="P320" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Life Patient Home Care</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr"/>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Sameer Ahmed</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>084455 58377</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>lifepatienthomecare@gmail.com</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>P-38, MARKET, Block P, Sector 12, Noida, Uttar Pradesh 201301</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr"/>
+      <c r="K321" t="inlineStr"/>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M321" t="inlineStr"/>
+      <c r="N321" t="inlineStr"/>
+      <c r="O321" t="inlineStr"/>
+      <c r="P321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Coloplast India Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr"/>
+      <c r="D322" t="inlineStr"/>
+      <c r="E322" t="inlineStr"/>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>0120 407 1300</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr"/>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>IGL Complex, 4th Floor (Right Wing), Tower 3, Plot No. – 2B, Sector 126, Noida, Uttar Pradesh 201304</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>06AAECC3545K1ZN</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>₹134.33 Crore</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M322" t="inlineStr"/>
+      <c r="N322" t="inlineStr"/>
+      <c r="O322" t="inlineStr"/>
+      <c r="P322" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>JK Engineering Works</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr"/>
+      <c r="D323" t="inlineStr"/>
+      <c r="E323" t="inlineStr"/>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>082850 26446</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>info@jkenggindia.com</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>C-30, Sector-57, Noida – 201301, Uttar Pradesh, India</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr"/>
+      <c r="K323" t="inlineStr"/>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr"/>
+      <c r="N323" t="inlineStr"/>
+      <c r="O323" t="inlineStr"/>
+      <c r="P323" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Kuvera Organics Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr"/>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Mr Atul Kumar Gupta</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>098102 28335</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr"/>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>G-2514, Prateek Edifice, Sector 107,Noida - 201304, Uttar Pradesh, India</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>09AAJCK3965G1Z5</t>
+        </is>
+      </c>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>₹8 Crores</t>
+        </is>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M324" t="inlineStr"/>
+      <c r="N324" t="inlineStr"/>
+      <c r="O324" t="inlineStr"/>
+      <c r="P324" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Innovation Meditech Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr"/>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Rajeev Agarwal</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>098110 58389</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>info@innovationmeditech.com</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>📍 B-6, Sector-88, Noida, UP – 201304</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>09AADCI3200N1ZM</t>
+        </is>
+      </c>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>₹39.62 Crore</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr"/>
+      <c r="N325" t="inlineStr"/>
+      <c r="O325" t="inlineStr"/>
+      <c r="P325" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>SpeechGears</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr"/>
+      <c r="D326" t="inlineStr"/>
+      <c r="E326" t="inlineStr"/>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>097735 57256</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>marketing@speechgears.com</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>SpeechGears India, B-17, Sector 60, Noida, U.P., 201301</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>09AAICG9712G1ZD</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>₹4.99 Crore</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr"/>
+      <c r="N326" t="inlineStr"/>
+      <c r="O326" t="inlineStr"/>
+      <c r="P326" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>MB Plastic Industries</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr"/>
+      <c r="D327" t="inlineStr"/>
+      <c r="E327" t="inlineStr"/>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>+911204985442</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>sales@mbplastic.com</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>B-75, Sector 83, Noida, UP 201305 IN</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>09ADFPJ7518J1Z9</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>Rs. 2.5 to 5 Crore Approx.</t>
+        </is>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M327" t="inlineStr"/>
+      <c r="N327" t="inlineStr"/>
+      <c r="O327" t="inlineStr"/>
+      <c r="P327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>OPTIAN HEALTHCARE PVT LTD</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr"/>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Reenu Gupta</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>011 6926 6203</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>info@optian.in</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>C25, Sector 8, Noida, Uttar Pradesh,201301</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr"/>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>₹1.19 Cr</t>
+        </is>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>unverified: declared industry could not be matched to a target segment; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M328" t="inlineStr"/>
+      <c r="N328" t="inlineStr"/>
+      <c r="O328" t="inlineStr"/>
+      <c r="P328" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Goodbooks</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>AB CONTRACTS</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr"/>
+      <c r="D329" t="inlineStr"/>
+      <c r="E329" t="inlineStr"/>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>011-46710423</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>helpdesk@tradeindia.com</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>148-B, Udyog Kendra-1, Ecotech-3, Greater Noida, Uttar Pradesh, 201303, India</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr"/>
+      <c r="K329" t="inlineStr"/>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>unverified: turnover unavailable; unverified: employee count unavailable</t>
+        </is>
+      </c>
+      <c r="M329" t="inlineStr"/>
+      <c r="N329" t="inlineStr"/>
+      <c r="O329" t="inlineStr"/>
+      <c r="P329" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P177"/>
+  <autoFilter ref="A1:P329"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>

</xml_diff>